<commit_message>
fix and fine tuning
</commit_message>
<xml_diff>
--- a/emission factors/other sources.xlsx
+++ b/emission factors/other sources.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365.sharepoint.com/sites/DENG-SESAM/Documenti condivisi/c-Research/b-Models/MARIO/Models/2026_JIE_Citterio_CFe/emission factors/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365.sharepoint.com/sites/DENG-SESAM/Documenti condivisi/c-Research/b-Models/MARIO/Models/2026_JIE_Citterio_CFe/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="8_{F5DCB09C-277A-2640-913B-E018972CB177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D15C8D35-9447-EA4E-A010-330E1A7E542F}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{F5DCB09C-277A-2640-913B-E018972CB177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0095022-CD22-C74C-A6C9-3AF6C024D3BE}"/>
   <bookViews>
-    <workbookView xWindow="-51200" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{EF5DED41-8CF6-EF48-85EB-50FED01B7F1A}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17660" xr2:uid="{EF5DED41-8CF6-EF48-85EB-50FED01B7F1A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3287" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3314" uniqueCount="61">
   <si>
     <t>Year</t>
   </si>
@@ -617,7 +617,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA30CEE6-49AA-0F4B-A88B-E50F140696EC}">
-  <dimension ref="A1:M466"/>
+  <dimension ref="A1:AB466"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.5" style="4" bestFit="1" customWidth="1"/>
@@ -13870,7 +13870,7 @@
         <v>120.920084354369</v>
       </c>
     </row>
-    <row r="401" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="401" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A401" s="2" t="s">
         <v>55</v>
       </c>
@@ -13909,7 +13909,7 @@
         <v>398.85565362854197</v>
       </c>
     </row>
-    <row r="402" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="402" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A402" s="2" t="s">
         <v>55</v>
       </c>
@@ -13948,7 +13948,7 @@
         <v>265.597704088613</v>
       </c>
     </row>
-    <row r="403" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="403" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A403" s="2" t="s">
         <v>55</v>
       </c>
@@ -13987,7 +13987,7 @@
         <v>400.54303635099501</v>
       </c>
     </row>
-    <row r="404" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="404" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A404" s="2" t="s">
         <v>55</v>
       </c>
@@ -14026,7 +14026,7 @@
         <v>3.2518309653554803E-2</v>
       </c>
     </row>
-    <row r="405" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="405" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A405" s="2" t="s">
         <v>55</v>
       </c>
@@ -14065,7 +14065,7 @@
         <v>1.81887536716836E-2</v>
       </c>
     </row>
-    <row r="406" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="406" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A406" s="2" t="s">
         <v>55</v>
       </c>
@@ -14104,7 +14104,7 @@
         <v>213.25902737675801</v>
       </c>
     </row>
-    <row r="407" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="407" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A407" s="2" t="s">
         <v>55</v>
       </c>
@@ -14143,7 +14143,7 @@
         <v>292.21637648995898</v>
       </c>
     </row>
-    <row r="408" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="408" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A408" s="2" t="s">
         <v>55</v>
       </c>
@@ -14182,7 +14182,7 @@
         <v>91.140581163508998</v>
       </c>
     </row>
-    <row r="409" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="409" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A409" s="2" t="s">
         <v>55</v>
       </c>
@@ -14221,7 +14221,7 @@
         <v>138.959741619006</v>
       </c>
     </row>
-    <row r="410" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="410" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A410" s="2" t="s">
         <v>55</v>
       </c>
@@ -14260,7 +14260,7 @@
         <v>359.44735757316602</v>
       </c>
     </row>
-    <row r="411" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="411" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A411" s="2" t="s">
         <v>55</v>
       </c>
@@ -14299,7 +14299,7 @@
         <v>441.13513896592002</v>
       </c>
     </row>
-    <row r="412" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="412" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A412" s="2" t="s">
         <v>49</v>
       </c>
@@ -14331,8 +14331,11 @@
       <c r="M412" s="3">
         <v>198.515256247341</v>
       </c>
-    </row>
-    <row r="413" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB412" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="413" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A413" s="2" t="s">
         <v>49</v>
       </c>
@@ -14364,8 +14367,11 @@
       <c r="M413" s="3">
         <v>188.047078175302</v>
       </c>
-    </row>
-    <row r="414" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB413" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="414" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A414" s="2" t="s">
         <v>49</v>
       </c>
@@ -14397,8 +14403,11 @@
       <c r="M414" s="3">
         <v>403.52162793620897</v>
       </c>
-    </row>
-    <row r="415" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB414" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="415" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A415" s="2" t="s">
         <v>49</v>
       </c>
@@ -14430,8 +14439,11 @@
       <c r="M415" s="3">
         <v>117.120823501161</v>
       </c>
-    </row>
-    <row r="416" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB415" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="416" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A416" s="2" t="s">
         <v>49</v>
       </c>
@@ -14463,8 +14475,11 @@
       <c r="M416" s="3">
         <v>528.34790778211004</v>
       </c>
-    </row>
-    <row r="417" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB416" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="417" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A417" s="2" t="s">
         <v>49</v>
       </c>
@@ -14496,8 +14511,11 @@
       <c r="M417" s="3">
         <v>630.86897814008103</v>
       </c>
-    </row>
-    <row r="418" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB417" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="418" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A418" s="2" t="s">
         <v>49</v>
       </c>
@@ -14529,8 +14547,11 @@
       <c r="M418" s="3">
         <v>174.41249057338399</v>
       </c>
-    </row>
-    <row r="419" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB418" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="419" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A419" s="2" t="s">
         <v>49</v>
       </c>
@@ -14562,8 +14583,11 @@
       <c r="M419" s="3">
         <v>211.54091233310501</v>
       </c>
-    </row>
-    <row r="420" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB419" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="420" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A420" s="2" t="s">
         <v>49</v>
       </c>
@@ -14595,8 +14619,11 @@
       <c r="M420" s="3">
         <v>289.99654573717601</v>
       </c>
-    </row>
-    <row r="421" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB420" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="421" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A421" s="2" t="s">
         <v>49</v>
       </c>
@@ -14628,8 +14655,11 @@
       <c r="M421" s="3">
         <v>187.84849540837999</v>
       </c>
-    </row>
-    <row r="422" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB421" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="422" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A422" s="2" t="s">
         <v>49</v>
       </c>
@@ -14661,8 +14691,11 @@
       <c r="M422" s="3">
         <v>103.06303413907</v>
       </c>
-    </row>
-    <row r="423" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB422" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="423" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A423" s="2" t="s">
         <v>49</v>
       </c>
@@ -14694,8 +14727,11 @@
       <c r="M423" s="3">
         <v>706.27989574635205</v>
       </c>
-    </row>
-    <row r="424" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB423" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="424" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A424" s="2" t="s">
         <v>49</v>
       </c>
@@ -14727,8 +14763,11 @@
       <c r="M424" s="3">
         <v>302.974747848672</v>
       </c>
-    </row>
-    <row r="425" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB424" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="425" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A425" s="2" t="s">
         <v>49</v>
       </c>
@@ -14760,8 +14799,11 @@
       <c r="M425" s="3">
         <v>265.832408375797</v>
       </c>
-    </row>
-    <row r="426" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB425" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="426" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A426" s="2" t="s">
         <v>49</v>
       </c>
@@ -14793,8 +14835,11 @@
       <c r="M426" s="3">
         <v>582.57225319718998</v>
       </c>
-    </row>
-    <row r="427" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB426" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="427" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A427" s="2" t="s">
         <v>49</v>
       </c>
@@ -14826,8 +14871,11 @@
       <c r="M427" s="3">
         <v>315.836631241161</v>
       </c>
-    </row>
-    <row r="428" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB427" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="428" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A428" s="2" t="s">
         <v>49</v>
       </c>
@@ -14859,8 +14907,11 @@
       <c r="M428" s="3">
         <v>64.043083488830206</v>
       </c>
-    </row>
-    <row r="429" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB428" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="429" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A429" s="2" t="s">
         <v>49</v>
       </c>
@@ -14892,8 +14943,11 @@
       <c r="M429" s="3">
         <v>172.77596669184501</v>
       </c>
-    </row>
-    <row r="430" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB429" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="430" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A430" s="2" t="s">
         <v>49</v>
       </c>
@@ -14925,8 +14979,11 @@
       <c r="M430" s="3">
         <v>148.87669157518201</v>
       </c>
-    </row>
-    <row r="431" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB430" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="431" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A431" s="2" t="s">
         <v>49</v>
       </c>
@@ -14958,8 +15015,11 @@
       <c r="M431" s="3">
         <v>518.856614102197</v>
       </c>
-    </row>
-    <row r="432" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB431" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="432" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A432" s="2" t="s">
         <v>49</v>
       </c>
@@ -14991,8 +15051,11 @@
       <c r="M432" s="3">
         <v>444.74019598317602</v>
       </c>
-    </row>
-    <row r="433" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB432" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="433" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A433" s="2" t="s">
         <v>49</v>
       </c>
@@ -15024,8 +15087,11 @@
       <c r="M433" s="3">
         <v>726.97762061901301</v>
       </c>
-    </row>
-    <row r="434" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB433" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="434" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A434" s="2" t="s">
         <v>49</v>
       </c>
@@ -15057,8 +15123,11 @@
       <c r="M434" s="3">
         <v>481.551182138954</v>
       </c>
-    </row>
-    <row r="435" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB434" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="435" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A435" s="2" t="s">
         <v>49</v>
       </c>
@@ -15090,8 +15159,11 @@
       <c r="M435" s="3">
         <v>369.79849815528399</v>
       </c>
-    </row>
-    <row r="436" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB435" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="436" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A436" s="2" t="s">
         <v>49</v>
       </c>
@@ -15123,8 +15195,11 @@
       <c r="M436" s="3">
         <v>28.600884300541299</v>
       </c>
-    </row>
-    <row r="437" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB436" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="437" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A437" s="2" t="s">
         <v>49</v>
       </c>
@@ -15156,8 +15231,11 @@
       <c r="M437" s="3">
         <v>335.98372041695001</v>
       </c>
-    </row>
-    <row r="438" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB437" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="438" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A438" s="2" t="s">
         <v>49</v>
       </c>
@@ -15189,8 +15267,11 @@
       <c r="M438" s="3">
         <v>267.39414781955702</v>
       </c>
-    </row>
-    <row r="439" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="AB438" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="439" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A439" s="2" t="s">
         <v>49</v>
       </c>
@@ -15223,7 +15304,7 @@
         <v>425.422489411051</v>
       </c>
     </row>
-    <row r="440" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="440" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A440" s="2" t="s">
         <v>38</v>
       </c>
@@ -15254,7 +15335,7 @@
         <v>315.53103420081197</v>
       </c>
     </row>
-    <row r="441" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="441" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A441" s="2" t="s">
         <v>38</v>
       </c>
@@ -15285,7 +15366,7 @@
         <v>217.128376783737</v>
       </c>
     </row>
-    <row r="442" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="442" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A442" s="2" t="s">
         <v>38</v>
       </c>
@@ -15316,7 +15397,7 @@
         <v>658.42801915841005</v>
       </c>
     </row>
-    <row r="443" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="443" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A443" s="2" t="s">
         <v>38</v>
       </c>
@@ -15347,7 +15428,7 @@
         <v>722.27949196409702</v>
       </c>
     </row>
-    <row r="444" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="444" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A444" s="2" t="s">
         <v>38</v>
       </c>
@@ -15378,7 +15459,7 @@
         <v>659.61877995075201</v>
       </c>
     </row>
-    <row r="445" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="445" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A445" s="2" t="s">
         <v>38</v>
       </c>
@@ -15409,7 +15490,7 @@
         <v>474.827287854926</v>
       </c>
     </row>
-    <row r="446" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="446" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A446" s="2" t="s">
         <v>38</v>
       </c>
@@ -15440,7 +15521,7 @@
         <v>140.55813143296101</v>
       </c>
     </row>
-    <row r="447" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="447" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A447" s="2" t="s">
         <v>38</v>
       </c>
@@ -15471,7 +15552,7 @@
         <v>1032.4652778131101</v>
       </c>
     </row>
-    <row r="448" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="448" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A448" s="2" t="s">
         <v>38</v>
       </c>
@@ -16066,15 +16147,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e">
@@ -16083,6 +16155,15 @@
     <TaxCatchAll xmlns="e67e9a88-35e1-4b39-8da9-a609eb308282" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -16347,26 +16428,26 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{256D0322-A8AB-48CD-9747-426763767878}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45D0A277-0A46-4490-85FB-A8106C6C8164}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="e67e9a88-35e1-4b39-8da9-a609eb308282"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45D0A277-0A46-4490-85FB-A8106C6C8164}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{256D0322-A8AB-48CD-9747-426763767878}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="5d44ae6a-e145-4c9d-94e7-ddf9cc58067e"/>
-    <ds:schemaRef ds:uri="e67e9a88-35e1-4b39-8da9-a609eb308282"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>